<commit_message>
feat: busqueda de noticias similares con multi-consulta y ediciones regionales
- news_finder reescrito: queries por titulo/entidades, fallback multi-edicion RSS (es-419 MX, es MX, es-419 US)
- exclusion de la noticia original por similitud de titulo >0.85 y URL
- analyzer.py y app.py pasan exclude_title/exclude_url/exclude_domain
- kanban: HU distribuidas por capitulos (Cap1 HU-01/02, Cap2 HU-03..07, Cap3 HU-08..29, Cap4 HU-30..39)
- gantt: Tony eliminado, 20 tareas repartidas (Marco 7, Luis 7, Ulises 6)
- docs de tesis: informe tecnico, modulos, glosario, usabilidad, format_apa, prompt presentacion
</commit_message>
<xml_diff>
--- a/tesis/Gantt_VERIFEX.xlsx
+++ b/tesis/Gantt_VERIFEX.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt VERIFEX" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gantt VERIFEX'!$A$1:$J$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gantt VERIFEX'!$A$1:$J$116</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,19 +85,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00B71C1C"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00E65100"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00C62828"/>
       <sz val="10"/>
     </font>
     <font>
@@ -106,7 +94,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -153,12 +141,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E3F2FD"/>
         <bgColor rgb="00E3F2FD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEBEE"/>
-        <bgColor rgb="00FFEBEE"/>
       </patternFill>
     </fill>
     <fill>
@@ -238,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -279,21 +261,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -302,8 +278,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -669,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J118"/>
+  <dimension ref="A1:J125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1091,9 +1065,9 @@
           <t>Herramientas de prueba: Vitest, Pytest, Playwright, Selenium</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F13" s="10" t="n">
@@ -1251,9 +1225,9 @@
           <t>Metricas de calidad, criterios de aceptacion y matriz de trazabilidad</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F17" s="10" t="n">
@@ -1411,9 +1385,9 @@
           <t>Plan maestro de pruebas y diseno de casos de prueba iniciales</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F21" s="10" t="n">
@@ -1477,42 +1451,42 @@
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="16" t="n"/>
-      <c r="B23" s="17" t="inlineStr">
+      <c r="A23" s="15" t="n"/>
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>Iteracion</t>
         </is>
       </c>
-      <c r="C23" s="17" t="inlineStr">
+      <c r="C23" s="16" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="D23" s="16" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>v0.1.0 - Requisitos, HU, marco teorico y plan de pruebas definidos</t>
         </is>
       </c>
-      <c r="E23" s="17" t="inlineStr">
+      <c r="E23" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F23" s="18" t="n">
+      <c r="F23" s="17" t="n">
         <v>45995</v>
       </c>
-      <c r="G23" s="18" t="n">
+      <c r="G23" s="17" t="n">
         <v>45996</v>
       </c>
-      <c r="H23" s="17" t="n">
+      <c r="H23" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="I23" s="17" t="inlineStr">
+      <c r="I23" s="16" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="J23" s="17" t="inlineStr">
+      <c r="J23" s="16" t="inlineStr">
         <is>
           <t>Lanzado</t>
         </is>
@@ -1552,9 +1526,9 @@
           <t>17</t>
         </is>
       </c>
-      <c r="J24" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -1725,9 +1699,9 @@
           <t>Diagramas UML: casos de uso, actividades, secuencia, clases, ER</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F30" s="10" t="n">
@@ -1885,9 +1859,9 @@
           <t>Datos de prueba y configuracion del entorno de validacion</t>
         </is>
       </c>
-      <c r="E34" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F34" s="10" t="n">
@@ -2045,9 +2019,9 @@
           <t>Casos de prueba detallados para scraper y extraccion de contenido</t>
         </is>
       </c>
-      <c r="E38" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F38" s="10" t="n">
@@ -2071,42 +2045,42 @@
       </c>
     </row>
     <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="16" t="n"/>
-      <c r="B39" s="17" t="inlineStr">
+      <c r="A39" s="15" t="n"/>
+      <c r="B39" s="16" t="inlineStr">
         <is>
           <t>Iteracion</t>
         </is>
       </c>
-      <c r="C39" s="17" t="inlineStr">
+      <c r="C39" s="16" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="D39" s="16" t="inlineStr">
+      <c r="D39" s="15" t="inlineStr">
         <is>
           <t>v0.2.0 - Diseno completo: arquitectura, prototipo navegable, diagramas UML y plan de pruebas detallado</t>
         </is>
       </c>
-      <c r="E39" s="17" t="inlineStr">
+      <c r="E39" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F39" s="18" t="n">
+      <c r="F39" s="17" t="n">
         <v>46034</v>
       </c>
-      <c r="G39" s="18" t="n">
+      <c r="G39" s="17" t="n">
         <v>46035</v>
       </c>
-      <c r="H39" s="17" t="n">
+      <c r="H39" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="I39" s="17" t="inlineStr">
+      <c r="I39" s="16" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="J39" s="17" t="inlineStr">
+      <c r="J39" s="16" t="inlineStr">
         <is>
           <t>Lanzado</t>
         </is>
@@ -2146,9 +2120,9 @@
           <t>29</t>
         </is>
       </c>
-      <c r="J40" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="J40" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -2319,9 +2293,9 @@
           <t>Configuracion de pruebas: pytest, vitest, jsdom, testing-library</t>
         </is>
       </c>
-      <c r="E46" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+      <c r="E46" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F46" s="10" t="n">
@@ -2479,9 +2453,9 @@
           <t>Pruebas del scraper y validacion de extraccion de contenido HTML</t>
         </is>
       </c>
-      <c r="E50" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+      <c r="E50" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F50" s="10" t="n">
@@ -2505,42 +2479,44 @@
       </c>
     </row>
     <row r="51" ht="24" customHeight="1">
-      <c r="A51" s="6" t="n"/>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="n">
-        <v>38</v>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>Llamadas a Groq API: call_groq, prompt engineering, parse_response</t>
-        </is>
-      </c>
-      <c r="E51" s="12" t="inlineStr">
-        <is>
-          <t>Marco</t>
-        </is>
-      </c>
-      <c r="F51" s="10" t="n">
+      <c r="A51" s="15" t="n"/>
+      <c r="B51" s="16" t="inlineStr">
+        <is>
+          <t>Iteracion</t>
+        </is>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="inlineStr">
+        <is>
+          <t>v0.3.0 - Scraper multi-estrategia funcional: cloudscraper, curl_cffi, requests y Playwright integrados y validados</t>
+        </is>
+      </c>
+      <c r="E51" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F51" s="17" t="n">
         <v>46062</v>
       </c>
-      <c r="G51" s="10" t="n">
-        <v>46074</v>
-      </c>
-      <c r="H51" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="I51" s="8" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="J51" s="11" t="inlineStr">
-        <is>
-          <t>Completado</t>
+      <c r="G51" s="17" t="n">
+        <v>46063</v>
+      </c>
+      <c r="H51" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I51" s="16" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="J51" s="16" t="inlineStr">
+        <is>
+          <t>Lanzado</t>
         </is>
       </c>
     </row>
@@ -2552,30 +2528,30 @@
         </is>
       </c>
       <c r="C52" s="8" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Manejo de estados (loading, error, results) y soporte bilingue ES/EN</t>
-        </is>
-      </c>
-      <c r="E52" s="13" t="inlineStr">
-        <is>
-          <t>Luis</t>
+          <t>Llamadas a Groq API: call_groq, prompt engineering, parse_response</t>
+        </is>
+      </c>
+      <c r="E52" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F52" s="10" t="n">
-        <v>46060</v>
+        <v>46062</v>
       </c>
       <c r="G52" s="10" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="H52" s="8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I52" s="8" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>34</t>
         </is>
       </c>
       <c r="J52" s="11" t="inlineStr">
@@ -2592,30 +2568,30 @@
         </is>
       </c>
       <c r="C53" s="8" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Actualizacion Capitulos 1-3 segun cambios de implementacion</t>
-        </is>
-      </c>
-      <c r="E53" s="14" t="inlineStr">
-        <is>
-          <t>Ulises</t>
+          <t>Manejo de estados (loading, error, results) y soporte bilingue ES/EN</t>
+        </is>
+      </c>
+      <c r="E53" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F53" s="10" t="n">
-        <v>46064</v>
+        <v>46060</v>
       </c>
       <c r="G53" s="10" t="n">
-        <v>46077</v>
+        <v>46071</v>
       </c>
       <c r="H53" s="8" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I53" s="8" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>35</t>
         </is>
       </c>
       <c r="J53" s="11" t="inlineStr">
@@ -2632,30 +2608,30 @@
         </is>
       </c>
       <c r="C54" s="8" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Pruebas de integracion scraper + Groq API con distintos tipos de URL</t>
-        </is>
-      </c>
-      <c r="E54" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+          <t>Actualizacion Capitulos 1-3 segun cambios de implementacion</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F54" s="10" t="n">
-        <v>46062</v>
+        <v>46064</v>
       </c>
       <c r="G54" s="10" t="n">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="H54" s="8" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I54" s="8" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>36</t>
         </is>
       </c>
       <c r="J54" s="11" t="inlineStr">
@@ -2672,30 +2648,30 @@
         </is>
       </c>
       <c r="C55" s="8" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Clasificador de credibilidad: 5 categorias, CREDIBLE_DOMAINS y override</t>
-        </is>
-      </c>
-      <c r="E55" s="12" t="inlineStr">
-        <is>
-          <t>Marco</t>
+          <t>Pruebas de integracion scraper + Groq API con distintos tipos de URL</t>
+        </is>
+      </c>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F55" s="10" t="n">
-        <v>46075</v>
+        <v>46062</v>
       </c>
       <c r="G55" s="10" t="n">
-        <v>46087</v>
+        <v>46074</v>
       </c>
       <c r="H55" s="8" t="n">
         <v>13</v>
       </c>
       <c r="I55" s="8" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>37</t>
         </is>
       </c>
       <c r="J55" s="11" t="inlineStr">
@@ -2712,30 +2688,30 @@
         </is>
       </c>
       <c r="C56" s="8" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Diseno visual cyberpunk: cuadricula, glitch, vignette CRT, scanlines</t>
-        </is>
-      </c>
-      <c r="E56" s="13" t="inlineStr">
-        <is>
-          <t>Luis</t>
+          <t>Clasificador de credibilidad: 5 categorias, CREDIBLE_DOMAINS y override</t>
+        </is>
+      </c>
+      <c r="E56" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F56" s="10" t="n">
-        <v>46072</v>
+        <v>46075</v>
       </c>
       <c r="G56" s="10" t="n">
-        <v>46083</v>
+        <v>46087</v>
       </c>
       <c r="H56" s="8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I56" s="8" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>38</t>
         </is>
       </c>
       <c r="J56" s="11" t="inlineStr">
@@ -2752,30 +2728,30 @@
         </is>
       </c>
       <c r="C57" s="8" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Tabla de resultados, analisis preliminar de datos e indice de tesis</t>
-        </is>
-      </c>
-      <c r="E57" s="14" t="inlineStr">
-        <is>
-          <t>Ulises</t>
+          <t>Diseno visual cyberpunk: cuadricula, glitch, vignette CRT, scanlines</t>
+        </is>
+      </c>
+      <c r="E57" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F57" s="10" t="n">
-        <v>46078</v>
+        <v>46072</v>
       </c>
       <c r="G57" s="10" t="n">
-        <v>46091</v>
+        <v>46083</v>
       </c>
       <c r="H57" s="8" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I57" s="8" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>39</t>
         </is>
       </c>
       <c r="J57" s="11" t="inlineStr">
@@ -2792,30 +2768,30 @@
         </is>
       </c>
       <c r="C58" s="8" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Pruebas de integracion frontend-backend con datos simulados y reales</t>
-        </is>
-      </c>
-      <c r="E58" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+          <t>Tabla de resultados, analisis preliminar de datos e indice de tesis</t>
+        </is>
+      </c>
+      <c r="E58" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F58" s="10" t="n">
-        <v>46075</v>
+        <v>46078</v>
       </c>
       <c r="G58" s="10" t="n">
-        <v>46087</v>
+        <v>46091</v>
       </c>
       <c r="H58" s="8" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I58" s="8" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J58" s="11" t="inlineStr">
@@ -2832,30 +2808,30 @@
         </is>
       </c>
       <c r="C59" s="8" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Busqueda de noticias similares: news_finder.py, Google News RSS</t>
-        </is>
-      </c>
-      <c r="E59" s="12" t="inlineStr">
-        <is>
-          <t>Marco</t>
+          <t>Pruebas de integracion frontend-backend con datos simulados y reales</t>
+        </is>
+      </c>
+      <c r="E59" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F59" s="10" t="n">
-        <v>46088</v>
+        <v>46075</v>
       </c>
       <c r="G59" s="10" t="n">
-        <v>46100</v>
+        <v>46087</v>
       </c>
       <c r="H59" s="8" t="n">
         <v>13</v>
       </c>
       <c r="I59" s="8" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>41</t>
         </is>
       </c>
       <c r="J59" s="11" t="inlineStr">
@@ -2865,42 +2841,44 @@
       </c>
     </row>
     <row r="60" ht="24" customHeight="1">
-      <c r="A60" s="6" t="n"/>
-      <c r="B60" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="n">
-        <v>47</v>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>Conexion frontend-backend via API REST (fetch /analyze + AbortController)</t>
-        </is>
-      </c>
-      <c r="E60" s="13" t="inlineStr">
-        <is>
-          <t>Luis</t>
-        </is>
-      </c>
-      <c r="F60" s="10" t="n">
-        <v>46084</v>
-      </c>
-      <c r="G60" s="10" t="n">
-        <v>46095</v>
-      </c>
-      <c r="H60" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I60" s="8" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="J60" s="11" t="inlineStr">
-        <is>
-          <t>Completado</t>
+      <c r="A60" s="15" t="n"/>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>Iteracion</t>
+        </is>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="D60" s="15" t="inlineStr">
+        <is>
+          <t>v0.4.0 - Clasificador de credibilidad, integracion frontend-backend y diseno cyberpunk completos</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F60" s="17" t="n">
+        <v>46088</v>
+      </c>
+      <c r="G60" s="17" t="n">
+        <v>46089</v>
+      </c>
+      <c r="H60" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I60" s="16" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="J60" s="16" t="inlineStr">
+        <is>
+          <t>Lanzado</t>
         </is>
       </c>
     </row>
@@ -2912,30 +2890,30 @@
         </is>
       </c>
       <c r="C61" s="8" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Referencias bibliograficas, anexos y plantilla oficial de tesis</t>
-        </is>
-      </c>
-      <c r="E61" s="14" t="inlineStr">
-        <is>
-          <t>Ulises</t>
+          <t>Busqueda de noticias similares: news_finder.py, Google News RSS</t>
+        </is>
+      </c>
+      <c r="E61" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F61" s="10" t="n">
-        <v>46092</v>
+        <v>46088</v>
       </c>
       <c r="G61" s="10" t="n">
-        <v>46105</v>
+        <v>46100</v>
       </c>
       <c r="H61" s="8" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I61" s="8" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J61" s="11" t="inlineStr">
@@ -2952,30 +2930,30 @@
         </is>
       </c>
       <c r="C62" s="8" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>Pruebas de regresion y deteccion de defectos en integracion continua</t>
-        </is>
-      </c>
-      <c r="E62" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+          <t>Conexion frontend-backend via API REST (fetch /analyze + AbortController)</t>
+        </is>
+      </c>
+      <c r="E62" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F62" s="10" t="n">
-        <v>46088</v>
+        <v>46084</v>
       </c>
       <c r="G62" s="10" t="n">
-        <v>46100</v>
+        <v>46095</v>
       </c>
       <c r="H62" s="8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I62" s="8" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J62" s="11" t="inlineStr">
@@ -2992,30 +2970,30 @@
         </is>
       </c>
       <c r="C63" s="8" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Article_type: 5 tipos y ajustes finales de clasificacion</t>
-        </is>
-      </c>
-      <c r="E63" s="12" t="inlineStr">
-        <is>
-          <t>Marco</t>
+          <t>Referencias bibliograficas, anexos y plantilla oficial de tesis</t>
+        </is>
+      </c>
+      <c r="E63" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F63" s="10" t="n">
-        <v>46101</v>
+        <v>46092</v>
       </c>
       <c r="G63" s="10" t="n">
-        <v>46111</v>
+        <v>46105</v>
       </c>
       <c r="H63" s="8" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I63" s="8" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>44</t>
         </is>
       </c>
       <c r="J63" s="11" t="inlineStr">
@@ -3032,11 +3010,11 @@
         </is>
       </c>
       <c r="C64" s="8" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>Manejo de errores de red, timeouts y UX de carga animada</t>
+          <t>Pruebas de regresion y deteccion de defectos en integracion continua</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
@@ -3045,17 +3023,17 @@
         </is>
       </c>
       <c r="F64" s="10" t="n">
-        <v>46096</v>
+        <v>46088</v>
       </c>
       <c r="G64" s="10" t="n">
-        <v>46105</v>
+        <v>46100</v>
       </c>
       <c r="H64" s="8" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I64" s="8" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>45</t>
         </is>
       </c>
       <c r="J64" s="11" t="inlineStr">
@@ -3072,30 +3050,30 @@
         </is>
       </c>
       <c r="C65" s="8" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Resultados parciales, graficas y tablas de visualizacion</t>
-        </is>
-      </c>
-      <c r="E65" s="14" t="inlineStr">
-        <is>
-          <t>Ulises</t>
+          <t>Article_type: 5 tipos y ajustes finales de clasificacion</t>
+        </is>
+      </c>
+      <c r="E65" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F65" s="10" t="n">
-        <v>46106</v>
+        <v>46101</v>
       </c>
       <c r="G65" s="10" t="n">
-        <v>46117</v>
+        <v>46111</v>
       </c>
       <c r="H65" s="8" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I65" s="8" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>46</t>
         </is>
       </c>
       <c r="J65" s="11" t="inlineStr">
@@ -3112,30 +3090,30 @@
         </is>
       </c>
       <c r="C66" s="8" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>Pruebas de aceptacion de usuario (UAT) con escenarios reales</t>
-        </is>
-      </c>
-      <c r="E66" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+          <t>Manejo de errores de red, timeouts y UX de carga animada</t>
+        </is>
+      </c>
+      <c r="E66" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F66" s="10" t="n">
-        <v>46101</v>
+        <v>46096</v>
       </c>
       <c r="G66" s="10" t="n">
-        <v>46111</v>
+        <v>46105</v>
       </c>
       <c r="H66" s="8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I66" s="8" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J66" s="11" t="inlineStr">
@@ -3145,44 +3123,42 @@
       </c>
     </row>
     <row r="67" ht="24" customHeight="1">
-      <c r="A67" s="16" t="n"/>
-      <c r="B67" s="17" t="inlineStr">
-        <is>
-          <t>Iteracion</t>
-        </is>
-      </c>
-      <c r="C67" s="17" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="D67" s="16" t="inlineStr">
-        <is>
-          <t>v0.5.0 - Desarrollo completo: scraper, IA, clasificador, news_finder, UI cyberpunk y pruebas de integracion</t>
-        </is>
-      </c>
-      <c r="E67" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F67" s="18" t="n">
-        <v>46112</v>
-      </c>
-      <c r="G67" s="18" t="n">
-        <v>46113</v>
-      </c>
-      <c r="H67" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="I67" s="17" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
-      </c>
-      <c r="J67" s="17" t="inlineStr">
-        <is>
-          <t>Lanzado</t>
+      <c r="A67" s="6" t="n"/>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>Resultados parciales, graficas y tablas de visualizacion</t>
+        </is>
+      </c>
+      <c r="E67" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
+        </is>
+      </c>
+      <c r="F67" s="10" t="n">
+        <v>46106</v>
+      </c>
+      <c r="G67" s="10" t="n">
+        <v>46117</v>
+      </c>
+      <c r="H67" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="I67" s="8" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="J67" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -3194,149 +3170,151 @@
         </is>
       </c>
       <c r="C68" s="8" t="n">
+        <v>53</v>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>Pruebas de aceptacion de usuario (UAT) con escenarios reales</t>
+        </is>
+      </c>
+      <c r="E68" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
+        </is>
+      </c>
+      <c r="F68" s="10" t="n">
+        <v>46101</v>
+      </c>
+      <c r="G68" s="10" t="n">
+        <v>46111</v>
+      </c>
+      <c r="H68" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="I68" s="8" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="J68" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="24" customHeight="1">
+      <c r="A69" s="15" t="n"/>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>Iteracion</t>
+        </is>
+      </c>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>v0.5.0 - Desarrollo completo: scraper, IA, clasificador, news_finder, UI cyberpunk y pruebas de integracion</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F69" s="17" t="n">
+        <v>46112</v>
+      </c>
+      <c r="G69" s="17" t="n">
+        <v>46113</v>
+      </c>
+      <c r="H69" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I69" s="16" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="J69" s="16" t="inlineStr">
+        <is>
+          <t>Lanzado</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="24" customHeight="1">
+      <c r="A70" s="6" t="n"/>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="n">
         <v>88</v>
       </c>
-      <c r="D68" s="6" t="inlineStr">
+      <c r="D70" s="6" t="inlineStr">
         <is>
           <t>Revision Ciclo 3: validacion del desarrollo completo y correcciones</t>
         </is>
       </c>
-      <c r="E68" s="9" t="inlineStr">
+      <c r="E70" s="9" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
       </c>
-      <c r="F68" s="10" t="n">
+      <c r="F70" s="10" t="n">
         <v>46112</v>
       </c>
-      <c r="G68" s="10" t="n">
+      <c r="G70" s="10" t="n">
         <v>46117</v>
       </c>
-      <c r="H68" s="8" t="n">
+      <c r="H70" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="I68" s="8" t="inlineStr">
+      <c r="I70" s="8" t="inlineStr">
         <is>
           <t>53</t>
         </is>
       </c>
-      <c r="J68" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="24" customHeight="1">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="J70" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="24" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>Ciclo 4: Validacion y Despliegue</t>
         </is>
       </c>
-      <c r="B69" s="3" t="n"/>
-      <c r="C69" s="3" t="n"/>
-      <c r="D69" s="3" t="n"/>
-      <c r="E69" s="3" t="n"/>
-      <c r="F69" s="3" t="n"/>
-      <c r="G69" s="3" t="n"/>
-      <c r="H69" s="3" t="n"/>
-      <c r="I69" s="3" t="n"/>
-      <c r="J69" s="3" t="n"/>
-    </row>
-    <row r="70" ht="24" customHeight="1">
-      <c r="A70" s="4" t="inlineStr">
+      <c r="B71" s="3" t="n"/>
+      <c r="C71" s="3" t="n"/>
+      <c r="D71" s="3" t="n"/>
+      <c r="E71" s="3" t="n"/>
+      <c r="F71" s="3" t="n"/>
+      <c r="G71" s="3" t="n"/>
+      <c r="H71" s="3" t="n"/>
+      <c r="I71" s="3" t="n"/>
+      <c r="J71" s="3" t="n"/>
+    </row>
+    <row r="72" ht="24" customHeight="1">
+      <c r="A72" s="4" t="inlineStr">
         <is>
           <t>Fase 4: Validacion y Despliegue</t>
         </is>
       </c>
-      <c r="B70" s="5" t="n"/>
-      <c r="C70" s="5" t="n"/>
-      <c r="D70" s="5" t="n"/>
-      <c r="E70" s="5" t="n"/>
-      <c r="F70" s="5" t="n"/>
-      <c r="G70" s="5" t="n"/>
-      <c r="H70" s="5" t="n"/>
-      <c r="I70" s="5" t="n"/>
-      <c r="J70" s="5" t="n"/>
-    </row>
-    <row r="71" ht="24" customHeight="1">
-      <c r="A71" s="6" t="n"/>
-      <c r="B71" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="n">
-        <v>54</v>
-      </c>
-      <c r="D71" s="6" t="inlineStr">
-        <is>
-          <t>Suite pruebas backend: 27 tests en server/test_analyzer.py (pytest)</t>
-        </is>
-      </c>
-      <c r="E71" s="12" t="inlineStr">
-        <is>
-          <t>Marco</t>
-        </is>
-      </c>
-      <c r="F71" s="10" t="n">
-        <v>46118</v>
-      </c>
-      <c r="G71" s="10" t="n">
-        <v>46130</v>
-      </c>
-      <c r="H71" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="I71" s="8" t="inlineStr">
-        <is>
-          <t>88</t>
-        </is>
-      </c>
-      <c r="J71" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="24" customHeight="1">
-      <c r="A72" s="6" t="n"/>
-      <c r="B72" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="n">
-        <v>55</v>
-      </c>
-      <c r="D72" s="6" t="inlineStr">
-        <is>
-          <t>Suite pruebas frontend: 52 tests con vitest + testing-library</t>
-        </is>
-      </c>
-      <c r="E72" s="13" t="inlineStr">
-        <is>
-          <t>Luis</t>
-        </is>
-      </c>
-      <c r="F72" s="10" t="n">
-        <v>46118</v>
-      </c>
-      <c r="G72" s="10" t="n">
-        <v>46129</v>
-      </c>
-      <c r="H72" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I72" s="8" t="inlineStr">
-        <is>
-          <t>88</t>
-        </is>
-      </c>
-      <c r="J72" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="B72" s="5" t="n"/>
+      <c r="C72" s="5" t="n"/>
+      <c r="D72" s="5" t="n"/>
+      <c r="E72" s="5" t="n"/>
+      <c r="F72" s="5" t="n"/>
+      <c r="G72" s="5" t="n"/>
+      <c r="H72" s="5" t="n"/>
+      <c r="I72" s="5" t="n"/>
+      <c r="J72" s="5" t="n"/>
     </row>
     <row r="73" ht="24" customHeight="1">
       <c r="A73" s="6" t="n"/>
@@ -3346,35 +3324,35 @@
         </is>
       </c>
       <c r="C73" s="8" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Resultados detallados y analisis de datos recopilados</t>
-        </is>
-      </c>
-      <c r="E73" s="14" t="inlineStr">
-        <is>
-          <t>Ulises</t>
+          <t>Suite pruebas backend: 27 tests en server/test_analyzer.py (pytest)</t>
+        </is>
+      </c>
+      <c r="E73" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F73" s="10" t="n">
         <v>46118</v>
       </c>
       <c r="G73" s="10" t="n">
-        <v>46131</v>
+        <v>46130</v>
       </c>
       <c r="H73" s="8" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I73" s="8" t="inlineStr">
         <is>
           <t>88</t>
         </is>
       </c>
-      <c r="J73" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="J73" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -3386,35 +3364,35 @@
         </is>
       </c>
       <c r="C74" s="8" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>Documentacion de pruebas: defectos, cobertura y metricas</t>
-        </is>
-      </c>
-      <c r="E74" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+          <t>Suite pruebas frontend: 52 tests con vitest + testing-library</t>
+        </is>
+      </c>
+      <c r="E74" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F74" s="10" t="n">
         <v>46118</v>
       </c>
       <c r="G74" s="10" t="n">
-        <v>46130</v>
+        <v>46129</v>
       </c>
       <c r="H74" s="8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I74" s="8" t="inlineStr">
         <is>
           <t>88</t>
         </is>
       </c>
-      <c r="J74" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="J74" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -3426,35 +3404,35 @@
         </is>
       </c>
       <c r="C75" s="8" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>Configuracion despliegue: Procfile, build.sh, CORS, gunicorn, Railway</t>
-        </is>
-      </c>
-      <c r="E75" s="12" t="inlineStr">
-        <is>
-          <t>Marco</t>
+          <t>Resultados detallados y analisis de datos recopilados</t>
+        </is>
+      </c>
+      <c r="E75" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F75" s="10" t="n">
+        <v>46118</v>
+      </c>
+      <c r="G75" s="10" t="n">
         <v>46131</v>
       </c>
-      <c r="G75" s="10" t="n">
-        <v>46143</v>
-      </c>
       <c r="H75" s="8" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I75" s="8" t="inlineStr">
         <is>
-          <t>54</t>
-        </is>
-      </c>
-      <c r="J75" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="J75" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -3466,75 +3444,77 @@
         </is>
       </c>
       <c r="C76" s="8" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
-          <t>Capturas del sistema: interfaz, resultados, errores, responsive</t>
-        </is>
-      </c>
-      <c r="E76" s="13" t="inlineStr">
-        <is>
-          <t>Luis</t>
+          <t>Documentacion de pruebas: defectos, cobertura y metricas</t>
+        </is>
+      </c>
+      <c r="E76" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F76" s="10" t="n">
+        <v>46118</v>
+      </c>
+      <c r="G76" s="10" t="n">
         <v>46130</v>
       </c>
-      <c r="G76" s="10" t="n">
-        <v>46141</v>
-      </c>
       <c r="H76" s="8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I76" s="8" t="inlineStr">
         <is>
-          <t>55</t>
-        </is>
-      </c>
-      <c r="J76" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="J76" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
     <row r="77" ht="24" customHeight="1">
-      <c r="A77" s="6" t="n"/>
-      <c r="B77" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C77" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="D77" s="6" t="inlineStr">
-        <is>
-          <t>Actualizacion bibliografia, graficas y tablas de visualizacion</t>
-        </is>
-      </c>
-      <c r="E77" s="14" t="inlineStr">
-        <is>
-          <t>Ulises</t>
-        </is>
-      </c>
-      <c r="F77" s="10" t="n">
+      <c r="A77" s="15" t="n"/>
+      <c r="B77" s="16" t="inlineStr">
+        <is>
+          <t>Iteracion</t>
+        </is>
+      </c>
+      <c r="C77" s="16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="D77" s="15" t="inlineStr">
+        <is>
+          <t>v0.6.0 - Suites completas de pruebas backend y frontend, resultados documentados y metricas de cobertura</t>
+        </is>
+      </c>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F77" s="17" t="n">
+        <v>46131</v>
+      </c>
+      <c r="G77" s="17" t="n">
         <v>46132</v>
       </c>
-      <c r="G77" s="10" t="n">
-        <v>46145</v>
-      </c>
-      <c r="H77" s="8" t="n">
-        <v>14</v>
-      </c>
-      <c r="I77" s="8" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-      <c r="J77" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H77" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I77" s="16" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="J77" s="16" t="inlineStr">
+        <is>
+          <t>Lanzado</t>
         </is>
       </c>
     </row>
@@ -3546,16 +3526,16 @@
         </is>
       </c>
       <c r="C78" s="8" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
-          <t>Validacion de seguridad: manejo errores, proteccion API key, estres</t>
-        </is>
-      </c>
-      <c r="E78" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+          <t>Configuracion despliegue: Procfile, build.sh, CORS, gunicorn, Railway</t>
+        </is>
+      </c>
+      <c r="E78" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F78" s="10" t="n">
@@ -3569,12 +3549,12 @@
       </c>
       <c r="I78" s="8" t="inlineStr">
         <is>
-          <t>57</t>
-        </is>
-      </c>
-      <c r="J78" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="J78" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -3586,35 +3566,35 @@
         </is>
       </c>
       <c r="C79" s="8" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Despliegue Railway → Render, dominio publico y SSL</t>
-        </is>
-      </c>
-      <c r="E79" s="12" t="inlineStr">
-        <is>
-          <t>Marco</t>
+          <t>Capturas del sistema: interfaz, resultados, errores, responsive</t>
+        </is>
+      </c>
+      <c r="E79" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F79" s="10" t="n">
-        <v>46144</v>
+        <v>46130</v>
       </c>
       <c r="G79" s="10" t="n">
-        <v>46156</v>
+        <v>46141</v>
       </c>
       <c r="H79" s="8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I79" s="8" t="inlineStr">
         <is>
-          <t>58</t>
-        </is>
-      </c>
-      <c r="J79" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="J79" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -3626,35 +3606,35 @@
         </is>
       </c>
       <c r="C80" s="8" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>Optimizacion frontend: lazy loading SimilarNews, code splitting</t>
-        </is>
-      </c>
-      <c r="E80" s="13" t="inlineStr">
-        <is>
-          <t>Luis</t>
+          <t>Actualizacion bibliografia, graficas y tablas de visualizacion</t>
+        </is>
+      </c>
+      <c r="E80" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F80" s="10" t="n">
-        <v>46142</v>
+        <v>46132</v>
       </c>
       <c r="G80" s="10" t="n">
-        <v>46153</v>
+        <v>46145</v>
       </c>
       <c r="H80" s="8" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I80" s="8" t="inlineStr">
         <is>
-          <t>59</t>
-        </is>
-      </c>
-      <c r="J80" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="J80" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -3666,117 +3646,117 @@
         </is>
       </c>
       <c r="C81" s="8" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Conclusiones preliminares y recomendaciones del proyecto</t>
-        </is>
-      </c>
-      <c r="E81" s="14" t="inlineStr">
-        <is>
-          <t>Ulises</t>
+          <t>Validacion de seguridad: manejo errores, proteccion API key, estres</t>
+        </is>
+      </c>
+      <c r="E81" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F81" s="10" t="n">
-        <v>46146</v>
+        <v>46131</v>
       </c>
       <c r="G81" s="10" t="n">
-        <v>46159</v>
+        <v>46143</v>
       </c>
       <c r="H81" s="8" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I81" s="8" t="inlineStr">
         <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="J81" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="J81" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
     <row r="82" ht="24" customHeight="1">
-      <c r="A82" s="6" t="n"/>
-      <c r="B82" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C82" s="8" t="n">
-        <v>65</v>
-      </c>
-      <c r="D82" s="6" t="inlineStr">
-        <is>
-          <t>Pruebas de rendimiento y carga en produccion (Render)</t>
-        </is>
-      </c>
-      <c r="E82" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
-        </is>
-      </c>
-      <c r="F82" s="10" t="n">
+      <c r="A82" s="15" t="n"/>
+      <c r="B82" s="16" t="inlineStr">
+        <is>
+          <t>Iteracion</t>
+        </is>
+      </c>
+      <c r="C82" s="16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="D82" s="15" t="inlineStr">
+        <is>
+          <t>v0.7.0 - Configuracion de despliegue, capturas del sistema, validacion de seguridad y bibliografia actualizada</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F82" s="17" t="n">
         <v>46144</v>
       </c>
-      <c r="G82" s="10" t="n">
+      <c r="G82" s="17" t="n">
+        <v>46145</v>
+      </c>
+      <c r="H82" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I82" s="16" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="J82" s="16" t="inlineStr">
+        <is>
+          <t>Lanzado</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="24" customHeight="1">
+      <c r="A83" s="6" t="n"/>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="n">
+        <v>62</v>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>Despliegue Railway → Render, dominio publico y SSL</t>
+        </is>
+      </c>
+      <c r="E83" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
+      <c r="F83" s="10" t="n">
+        <v>46144</v>
+      </c>
+      <c r="G83" s="10" t="n">
         <v>46156</v>
       </c>
-      <c r="H82" s="8" t="n">
+      <c r="H83" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="I82" s="8" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="J82" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="24" customHeight="1">
-      <c r="A83" s="16" t="n"/>
-      <c r="B83" s="17" t="inlineStr">
-        <is>
-          <t>Iteracion</t>
-        </is>
-      </c>
-      <c r="C83" s="17" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="D83" s="16" t="inlineStr">
-        <is>
-          <t>v1.0.0 - Version estable desplegada en Render con suite completa de pruebas y dominio publico</t>
-        </is>
-      </c>
-      <c r="E83" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F83" s="18" t="n">
-        <v>46157</v>
-      </c>
-      <c r="G83" s="18" t="n">
-        <v>46158</v>
-      </c>
-      <c r="H83" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="I83" s="17" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
-      </c>
-      <c r="J83" s="17" t="inlineStr">
-        <is>
-          <t>Lanzado</t>
+      <c r="I83" s="8" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="J83" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -3788,107 +3768,157 @@
         </is>
       </c>
       <c r="C84" s="8" t="n">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="D84" s="6" t="inlineStr">
         <is>
-          <t>Revision Ciclo 4: validacion del despliegue, pruebas y rendimiento</t>
-        </is>
-      </c>
-      <c r="E84" s="9" t="inlineStr">
-        <is>
-          <t>Todos</t>
+          <t>Optimizacion frontend: lazy loading SimilarNews, code splitting</t>
+        </is>
+      </c>
+      <c r="E84" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F84" s="10" t="n">
+        <v>46142</v>
+      </c>
+      <c r="G84" s="10" t="n">
+        <v>46153</v>
+      </c>
+      <c r="H84" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="I84" s="8" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="J84" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="24" customHeight="1">
+      <c r="A85" s="6" t="n"/>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>Conclusiones preliminares y recomendaciones del proyecto</t>
+        </is>
+      </c>
+      <c r="E85" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
+        </is>
+      </c>
+      <c r="F85" s="10" t="n">
+        <v>46146</v>
+      </c>
+      <c r="G85" s="10" t="n">
+        <v>46159</v>
+      </c>
+      <c r="H85" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="I85" s="8" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="J85" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="24" customHeight="1">
+      <c r="A86" s="6" t="n"/>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>Pruebas de rendimiento y carga en produccion (Render)</t>
+        </is>
+      </c>
+      <c r="E86" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
+      <c r="F86" s="10" t="n">
+        <v>46144</v>
+      </c>
+      <c r="G86" s="10" t="n">
+        <v>46156</v>
+      </c>
+      <c r="H86" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="I86" s="8" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="J86" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="24" customHeight="1">
+      <c r="A87" s="15" t="n"/>
+      <c r="B87" s="16" t="inlineStr">
+        <is>
+          <t>Iteracion</t>
+        </is>
+      </c>
+      <c r="C87" s="16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="D87" s="15" t="inlineStr">
+        <is>
+          <t>v0.8.0 - Version desplegada en Render con dominio publico, SSL, optimizaciones frontend y pruebas de rendimiento</t>
+        </is>
+      </c>
+      <c r="E87" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F87" s="17" t="n">
         <v>46157</v>
       </c>
-      <c r="G84" s="10" t="n">
-        <v>46162</v>
-      </c>
-      <c r="H84" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="I84" s="8" t="inlineStr">
+      <c r="G87" s="17" t="n">
+        <v>46158</v>
+      </c>
+      <c r="H87" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I87" s="16" t="inlineStr">
         <is>
           <t>65</t>
         </is>
       </c>
-      <c r="J84" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="24" customHeight="1">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>Ciclo 5: Resultados y Documentacion Final</t>
-        </is>
-      </c>
-      <c r="B85" s="3" t="n"/>
-      <c r="C85" s="3" t="n"/>
-      <c r="D85" s="3" t="n"/>
-      <c r="E85" s="3" t="n"/>
-      <c r="F85" s="3" t="n"/>
-      <c r="G85" s="3" t="n"/>
-      <c r="H85" s="3" t="n"/>
-      <c r="I85" s="3" t="n"/>
-      <c r="J85" s="3" t="n"/>
-    </row>
-    <row r="86" ht="24" customHeight="1">
-      <c r="A86" s="4" t="inlineStr">
-        <is>
-          <t>Fase 5: Resultados y Documentacion Final</t>
-        </is>
-      </c>
-      <c r="B86" s="5" t="n"/>
-      <c r="C86" s="5" t="n"/>
-      <c r="D86" s="5" t="n"/>
-      <c r="E86" s="5" t="n"/>
-      <c r="F86" s="5" t="n"/>
-      <c r="G86" s="5" t="n"/>
-      <c r="H86" s="5" t="n"/>
-      <c r="I86" s="5" t="n"/>
-      <c r="J86" s="5" t="n"/>
-    </row>
-    <row r="87" ht="24" customHeight="1">
-      <c r="A87" s="6" t="n"/>
-      <c r="B87" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="n">
-        <v>66</v>
-      </c>
-      <c r="D87" s="6" t="inlineStr">
-        <is>
-          <t>Analisis con URLs reales: Milenio, Reforma, Aristegui, estafas</t>
-        </is>
-      </c>
-      <c r="E87" s="12" t="inlineStr">
-        <is>
-          <t>Marco</t>
-        </is>
-      </c>
-      <c r="F87" s="10" t="n">
-        <v>46163</v>
-      </c>
-      <c r="G87" s="10" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H87" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="I87" s="8" t="inlineStr">
-        <is>
-          <t>89</t>
-        </is>
-      </c>
-      <c r="J87" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="J87" s="16" t="inlineStr">
+        <is>
+          <t>Lanzado</t>
         </is>
       </c>
     </row>
@@ -3900,157 +3930,111 @@
         </is>
       </c>
       <c r="C88" s="8" t="n">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="D88" s="6" t="inlineStr">
         <is>
-          <t>Diseno responsive: ajustes layout para movil, tablet y escritorio</t>
-        </is>
-      </c>
-      <c r="E88" s="13" t="inlineStr">
-        <is>
-          <t>Luis</t>
+          <t>Revision Ciclo 4: validacion del despliegue, pruebas y rendimiento</t>
+        </is>
+      </c>
+      <c r="E88" s="9" t="inlineStr">
+        <is>
+          <t>Todos</t>
         </is>
       </c>
       <c r="F88" s="10" t="n">
+        <v>46157</v>
+      </c>
+      <c r="G88" s="10" t="n">
+        <v>46162</v>
+      </c>
+      <c r="H88" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="I88" s="8" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="J88" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="24" customHeight="1">
+      <c r="A89" s="15" t="n"/>
+      <c r="B89" s="16" t="inlineStr">
+        <is>
+          <t>Iteracion</t>
+        </is>
+      </c>
+      <c r="C89" s="16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="D89" s="15" t="inlineStr">
+        <is>
+          <t>v0.9.0 - Validacion post-despliegue completada, rendimiento verificado y ajustes finales de integracion</t>
+        </is>
+      </c>
+      <c r="E89" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F89" s="17" t="n">
         <v>46163</v>
       </c>
-      <c r="G88" s="10" t="n">
-        <v>46174</v>
-      </c>
-      <c r="H88" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I88" s="8" t="inlineStr">
+      <c r="G89" s="17" t="n">
+        <v>46164</v>
+      </c>
+      <c r="H89" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I89" s="16" t="inlineStr">
         <is>
           <t>89</t>
         </is>
       </c>
-      <c r="J88" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="24" customHeight="1">
-      <c r="A89" s="6" t="n"/>
-      <c r="B89" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C89" s="8" t="n">
-        <v>68</v>
-      </c>
-      <c r="D89" s="6" t="inlineStr">
-        <is>
-          <t>Capitulo 5: Resultados, pruebas, analisis de datos y conclusiones</t>
-        </is>
-      </c>
-      <c r="E89" s="14" t="inlineStr">
-        <is>
-          <t>Ulises</t>
-        </is>
-      </c>
-      <c r="F89" s="10" t="n">
-        <v>46163</v>
-      </c>
-      <c r="G89" s="10" t="n">
-        <v>46176</v>
-      </c>
-      <c r="H89" s="8" t="n">
-        <v>14</v>
-      </c>
-      <c r="I89" s="8" t="inlineStr">
-        <is>
-          <t>89</t>
-        </is>
-      </c>
-      <c r="J89" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="J89" s="16" t="inlineStr">
+        <is>
+          <t>Lanzado</t>
         </is>
       </c>
     </row>
     <row r="90" ht="24" customHeight="1">
-      <c r="A90" s="6" t="n"/>
-      <c r="B90" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C90" s="8" t="n">
-        <v>69</v>
-      </c>
-      <c r="D90" s="6" t="inlineStr">
-        <is>
-          <t>Pruebas de regresion post-despliegue y verificacion funcional</t>
-        </is>
-      </c>
-      <c r="E90" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
-        </is>
-      </c>
-      <c r="F90" s="10" t="n">
-        <v>46163</v>
-      </c>
-      <c r="G90" s="10" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H90" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="I90" s="8" t="inlineStr">
-        <is>
-          <t>89</t>
-        </is>
-      </c>
-      <c r="J90" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Ciclo 5: Resultados y Documentacion Final</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="n"/>
+      <c r="C90" s="3" t="n"/>
+      <c r="D90" s="3" t="n"/>
+      <c r="E90" s="3" t="n"/>
+      <c r="F90" s="3" t="n"/>
+      <c r="G90" s="3" t="n"/>
+      <c r="H90" s="3" t="n"/>
+      <c r="I90" s="3" t="n"/>
+      <c r="J90" s="3" t="n"/>
     </row>
     <row r="91" ht="24" customHeight="1">
-      <c r="A91" s="6" t="n"/>
-      <c r="B91" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C91" s="8" t="n">
-        <v>70</v>
-      </c>
-      <c r="D91" s="6" t="inlineStr">
-        <is>
-          <t>Correccion errores: timeouts, override de dominios, edge cases URLs</t>
-        </is>
-      </c>
-      <c r="E91" s="12" t="inlineStr">
-        <is>
-          <t>Marco</t>
-        </is>
-      </c>
-      <c r="F91" s="10" t="n">
-        <v>46176</v>
-      </c>
-      <c r="G91" s="10" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H91" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="I91" s="8" t="inlineStr">
-        <is>
-          <t>66</t>
-        </is>
-      </c>
-      <c r="J91" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>Fase 5: Resultados y Documentacion Final</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="n"/>
+      <c r="C91" s="5" t="n"/>
+      <c r="D91" s="5" t="n"/>
+      <c r="E91" s="5" t="n"/>
+      <c r="F91" s="5" t="n"/>
+      <c r="G91" s="5" t="n"/>
+      <c r="H91" s="5" t="n"/>
+      <c r="I91" s="5" t="n"/>
+      <c r="J91" s="5" t="n"/>
     </row>
     <row r="92" ht="24" customHeight="1">
       <c r="A92" s="6" t="n"/>
@@ -4060,35 +4044,35 @@
         </is>
       </c>
       <c r="C92" s="8" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D92" s="6" t="inlineStr">
         <is>
-          <t>Manual de usuario completo y guia de uso del sistema</t>
-        </is>
-      </c>
-      <c r="E92" s="13" t="inlineStr">
-        <is>
-          <t>Luis</t>
+          <t>Analisis con URLs reales: Milenio, Reforma, Aristegui, estafas</t>
+        </is>
+      </c>
+      <c r="E92" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F92" s="10" t="n">
+        <v>46163</v>
+      </c>
+      <c r="G92" s="10" t="n">
         <v>46175</v>
       </c>
-      <c r="G92" s="10" t="n">
-        <v>46186</v>
-      </c>
       <c r="H92" s="8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I92" s="8" t="inlineStr">
         <is>
-          <t>67</t>
-        </is>
-      </c>
-      <c r="J92" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="J92" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -4100,35 +4084,35 @@
         </is>
       </c>
       <c r="C93" s="8" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Introduccion, resumen y abstract en espanol e ingles</t>
-        </is>
-      </c>
-      <c r="E93" s="14" t="inlineStr">
-        <is>
-          <t>Ulises</t>
+          <t>Diseno responsive: ajustes layout para movil, tablet y escritorio</t>
+        </is>
+      </c>
+      <c r="E93" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F93" s="10" t="n">
-        <v>46177</v>
+        <v>46163</v>
       </c>
       <c r="G93" s="10" t="n">
-        <v>46190</v>
+        <v>46174</v>
       </c>
       <c r="H93" s="8" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I93" s="8" t="inlineStr">
         <is>
-          <t>68</t>
-        </is>
-      </c>
-      <c r="J93" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="J93" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -4140,35 +4124,35 @@
         </is>
       </c>
       <c r="C94" s="8" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D94" s="6" t="inlineStr">
         <is>
-          <t>Documentacion tecnica: manual API, arquitectura, despliegue</t>
-        </is>
-      </c>
-      <c r="E94" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+          <t>Capitulo 5: Resultados, pruebas, analisis de datos y conclusiones</t>
+        </is>
+      </c>
+      <c r="E94" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F94" s="10" t="n">
+        <v>46163</v>
+      </c>
+      <c r="G94" s="10" t="n">
         <v>46176</v>
       </c>
-      <c r="G94" s="10" t="n">
-        <v>46188</v>
-      </c>
       <c r="H94" s="8" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I94" s="8" t="inlineStr">
         <is>
-          <t>69</t>
-        </is>
-      </c>
-      <c r="J94" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="J94" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -4180,75 +4164,77 @@
         </is>
       </c>
       <c r="C95" s="8" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Verificacion funcionalidad, pruebas de humo y validacion URLs reales</t>
-        </is>
-      </c>
-      <c r="E95" s="12" t="inlineStr">
-        <is>
-          <t>Marco</t>
+          <t>Pruebas de regresion post-despliegue y verificacion funcional</t>
+        </is>
+      </c>
+      <c r="E95" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F95" s="10" t="n">
-        <v>46189</v>
+        <v>46163</v>
       </c>
       <c r="G95" s="10" t="n">
-        <v>46201</v>
+        <v>46175</v>
       </c>
       <c r="H95" s="8" t="n">
         <v>13</v>
       </c>
       <c r="I95" s="8" t="inlineStr">
         <is>
-          <t>70</t>
-        </is>
-      </c>
-      <c r="J95" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="J95" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
     <row r="96" ht="24" customHeight="1">
-      <c r="A96" s="6" t="n"/>
-      <c r="B96" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="n">
-        <v>75</v>
-      </c>
-      <c r="D96" s="6" t="inlineStr">
-        <is>
-          <t>Maquetacion tesis Word: estilos, indices, tablas de contenido</t>
-        </is>
-      </c>
-      <c r="E96" s="13" t="inlineStr">
-        <is>
-          <t>Luis</t>
-        </is>
-      </c>
-      <c r="F96" s="10" t="n">
-        <v>46187</v>
-      </c>
-      <c r="G96" s="10" t="n">
-        <v>46198</v>
-      </c>
-      <c r="H96" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I96" s="8" t="inlineStr">
-        <is>
-          <t>71</t>
-        </is>
-      </c>
-      <c r="J96" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="A96" s="15" t="n"/>
+      <c r="B96" s="16" t="inlineStr">
+        <is>
+          <t>Iteracion</t>
+        </is>
+      </c>
+      <c r="C96" s="16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="D96" s="15" t="inlineStr">
+        <is>
+          <t>v0.10.0 - Analisis con URLs reales, diseno responsive, resultados preliminares y pruebas de regresion post-despliegue</t>
+        </is>
+      </c>
+      <c r="E96" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F96" s="17" t="n">
+        <v>46176</v>
+      </c>
+      <c r="G96" s="17" t="n">
+        <v>46177</v>
+      </c>
+      <c r="H96" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I96" s="16" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="J96" s="16" t="inlineStr">
+        <is>
+          <t>Lanzado</t>
         </is>
       </c>
     </row>
@@ -4260,35 +4246,35 @@
         </is>
       </c>
       <c r="C97" s="8" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>Revision ortografia, gramatica y consistencia de la tesis</t>
-        </is>
-      </c>
-      <c r="E97" s="14" t="inlineStr">
-        <is>
-          <t>Ulises</t>
+          <t>Correccion errores: timeouts, override de dominios, edge cases URLs</t>
+        </is>
+      </c>
+      <c r="E97" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>46191</v>
+        <v>46176</v>
       </c>
       <c r="G97" s="10" t="n">
-        <v>46204</v>
+        <v>46188</v>
       </c>
       <c r="H97" s="8" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I97" s="8" t="inlineStr">
         <is>
-          <t>72</t>
-        </is>
-      </c>
-      <c r="J97" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="J97" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -4300,35 +4286,35 @@
         </is>
       </c>
       <c r="C98" s="8" t="n">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D98" s="6" t="inlineStr">
         <is>
-          <t>Correcciones estilo, citas y normas institucionales</t>
-        </is>
-      </c>
-      <c r="E98" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+          <t>Manual de usuario completo y guia de uso del sistema</t>
+        </is>
+      </c>
+      <c r="E98" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F98" s="10" t="n">
-        <v>46189</v>
+        <v>46175</v>
       </c>
       <c r="G98" s="10" t="n">
-        <v>46201</v>
+        <v>46186</v>
       </c>
       <c r="H98" s="8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I98" s="8" t="inlineStr">
         <is>
-          <t>73</t>
-        </is>
-      </c>
-      <c r="J98" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="J98" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -4340,35 +4326,35 @@
         </is>
       </c>
       <c r="C99" s="8" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>Revision tecnica tesis: datos, consistencia Capitulos 4-5 y codigo</t>
-        </is>
-      </c>
-      <c r="E99" s="12" t="inlineStr">
-        <is>
-          <t>Marco</t>
+          <t>Introduccion, resumen y abstract en espanol e ingles</t>
+        </is>
+      </c>
+      <c r="E99" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>46202</v>
+        <v>46177</v>
       </c>
       <c r="G99" s="10" t="n">
-        <v>46220</v>
+        <v>46190</v>
       </c>
       <c r="H99" s="8" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="I99" s="8" t="inlineStr">
         <is>
-          <t>74</t>
-        </is>
-      </c>
-      <c r="J99" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="J99" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -4380,75 +4366,77 @@
         </is>
       </c>
       <c r="C100" s="8" t="n">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="D100" s="6" t="inlineStr">
         <is>
-          <t>Material presentacion defensa: diapositivas, demo y resultados</t>
-        </is>
-      </c>
-      <c r="E100" s="13" t="inlineStr">
-        <is>
-          <t>Luis</t>
+          <t>Documentacion tecnica: manual API, arquitectura, despliegue</t>
+        </is>
+      </c>
+      <c r="E100" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F100" s="10" t="n">
-        <v>46199</v>
+        <v>46176</v>
       </c>
       <c r="G100" s="10" t="n">
-        <v>46216</v>
+        <v>46188</v>
       </c>
       <c r="H100" s="8" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I100" s="8" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="J100" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="J100" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
     <row r="101" ht="24" customHeight="1">
-      <c r="A101" s="6" t="n"/>
-      <c r="B101" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C101" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="D101" s="6" t="inlineStr">
-        <is>
-          <t>Correcciones finales segun retroalimentacion del asesor</t>
-        </is>
-      </c>
-      <c r="E101" s="14" t="inlineStr">
-        <is>
-          <t>Ulises</t>
-        </is>
-      </c>
-      <c r="F101" s="10" t="n">
-        <v>46205</v>
-      </c>
-      <c r="G101" s="10" t="n">
-        <v>46224</v>
-      </c>
-      <c r="H101" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="I101" s="8" t="inlineStr">
-        <is>
-          <t>76</t>
-        </is>
-      </c>
-      <c r="J101" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="A101" s="15" t="n"/>
+      <c r="B101" s="16" t="inlineStr">
+        <is>
+          <t>Iteracion</t>
+        </is>
+      </c>
+      <c r="C101" s="16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="D101" s="15" t="inlineStr">
+        <is>
+          <t>v1.0.0 - Documentacion completa, manuales, resultados consolidados y version estable del sistema</t>
+        </is>
+      </c>
+      <c r="E101" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F101" s="17" t="n">
+        <v>46189</v>
+      </c>
+      <c r="G101" s="17" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H101" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I101" s="16" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="J101" s="16" t="inlineStr">
+        <is>
+          <t>Lanzado</t>
         </is>
       </c>
     </row>
@@ -4460,35 +4448,35 @@
         </is>
       </c>
       <c r="C102" s="8" t="n">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="D102" s="6" t="inlineStr">
         <is>
-          <t>Preparacion defensa tesis: diapositivas, demo en vivo y Q&amp;A</t>
-        </is>
-      </c>
-      <c r="E102" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
+          <t>Verificacion funcionalidad, pruebas de humo y validacion URLs reales</t>
+        </is>
+      </c>
+      <c r="E102" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
         </is>
       </c>
       <c r="F102" s="10" t="n">
-        <v>46202</v>
+        <v>46189</v>
       </c>
       <c r="G102" s="10" t="n">
-        <v>46220</v>
+        <v>46201</v>
       </c>
       <c r="H102" s="8" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="I102" s="8" t="inlineStr">
         <is>
-          <t>77</t>
-        </is>
-      </c>
-      <c r="J102" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="J102" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -4500,35 +4488,35 @@
         </is>
       </c>
       <c r="C103" s="8" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>Revision y aprobacion del asesor: validacion final tesis y sistema</t>
-        </is>
-      </c>
-      <c r="E103" s="9" t="inlineStr">
-        <is>
-          <t>Todos</t>
+          <t>Maquetacion tesis Word: estilos, indices, tablas de contenido</t>
+        </is>
+      </c>
+      <c r="E103" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
         </is>
       </c>
       <c r="F103" s="10" t="n">
-        <v>46221</v>
+        <v>46187</v>
       </c>
       <c r="G103" s="10" t="n">
-        <v>46233</v>
+        <v>46198</v>
       </c>
       <c r="H103" s="8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I103" s="8" t="inlineStr">
         <is>
-          <t>78</t>
-        </is>
-      </c>
-      <c r="J103" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="J103" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -4540,35 +4528,35 @@
         </is>
       </c>
       <c r="C104" s="8" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D104" s="6" t="inlineStr">
         <is>
-          <t>Cierre proyecto: limpieza codigo, README, tag v1.2.0 en git</t>
-        </is>
-      </c>
-      <c r="E104" s="12" t="inlineStr">
-        <is>
-          <t>Marco</t>
+          <t>Revision ortografia, gramatica y consistencia de la tesis</t>
+        </is>
+      </c>
+      <c r="E104" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F104" s="10" t="n">
-        <v>46234</v>
+        <v>46191</v>
       </c>
       <c r="G104" s="10" t="n">
-        <v>46254</v>
+        <v>46204</v>
       </c>
       <c r="H104" s="8" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="I104" s="8" t="inlineStr">
         <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="J104" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="J104" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
@@ -4580,75 +4568,77 @@
         </is>
       </c>
       <c r="C105" s="8" t="n">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>PDF final de tesis (TESIS_VERIFEX.pdf) con formato definitivo</t>
-        </is>
-      </c>
-      <c r="E105" s="13" t="inlineStr">
-        <is>
-          <t>Luis</t>
+          <t>Correcciones estilo, citas y normas institucionales</t>
+        </is>
+      </c>
+      <c r="E105" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
         </is>
       </c>
       <c r="F105" s="10" t="n">
-        <v>46234</v>
+        <v>46189</v>
       </c>
       <c r="G105" s="10" t="n">
-        <v>46253</v>
+        <v>46201</v>
       </c>
       <c r="H105" s="8" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="I105" s="8" t="inlineStr">
         <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="J105" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="J105" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
         </is>
       </c>
     </row>
     <row r="106" ht="24" customHeight="1">
-      <c r="A106" s="6" t="n"/>
-      <c r="B106" s="7" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="C106" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="D106" s="6" t="inlineStr">
-        <is>
-          <t>Revision final y validacion de entrega segun requisitos</t>
-        </is>
-      </c>
-      <c r="E106" s="14" t="inlineStr">
-        <is>
-          <t>Ulises</t>
-        </is>
-      </c>
-      <c r="F106" s="10" t="n">
-        <v>46234</v>
-      </c>
-      <c r="G106" s="10" t="n">
-        <v>46255</v>
-      </c>
-      <c r="H106" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="I106" s="8" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="J106" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="A106" s="15" t="n"/>
+      <c r="B106" s="16" t="inlineStr">
+        <is>
+          <t>Iteracion</t>
+        </is>
+      </c>
+      <c r="C106" s="16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="D106" s="15" t="inlineStr">
+        <is>
+          <t>v1.1.0 - Revisiones finales, verificacion funcional, maquetacion de tesis y correcciones de estilo</t>
+        </is>
+      </c>
+      <c r="E106" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F106" s="17" t="n">
+        <v>46202</v>
+      </c>
+      <c r="G106" s="17" t="n">
+        <v>46203</v>
+      </c>
+      <c r="H106" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I106" s="16" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="J106" s="16" t="inlineStr">
+        <is>
+          <t>Lanzado</t>
         </is>
       </c>
     </row>
@@ -4660,181 +4650,490 @@
         </is>
       </c>
       <c r="C107" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="D107" s="6" t="inlineStr">
+        <is>
+          <t>Revision tecnica tesis: datos, consistencia Capitulos 4-5 y codigo</t>
+        </is>
+      </c>
+      <c r="E107" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
+      <c r="F107" s="10" t="n">
+        <v>46202</v>
+      </c>
+      <c r="G107" s="10" t="n">
+        <v>46220</v>
+      </c>
+      <c r="H107" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="I107" s="8" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="J107" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="24" customHeight="1">
+      <c r="A108" s="6" t="n"/>
+      <c r="B108" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>Material presentacion defensa: diapositivas, demo y resultados</t>
+        </is>
+      </c>
+      <c r="E108" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="F108" s="10" t="n">
+        <v>46199</v>
+      </c>
+      <c r="G108" s="10" t="n">
+        <v>46216</v>
+      </c>
+      <c r="H108" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="I108" s="8" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="J108" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="24" customHeight="1">
+      <c r="A109" s="6" t="n"/>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="D109" s="6" t="inlineStr">
+        <is>
+          <t>Correcciones finales segun retroalimentacion del asesor</t>
+        </is>
+      </c>
+      <c r="E109" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
+        </is>
+      </c>
+      <c r="F109" s="10" t="n">
+        <v>46205</v>
+      </c>
+      <c r="G109" s="10" t="n">
+        <v>46224</v>
+      </c>
+      <c r="H109" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I109" s="8" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="J109" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="24" customHeight="1">
+      <c r="A110" s="6" t="n"/>
+      <c r="B110" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="D110" s="6" t="inlineStr">
+        <is>
+          <t>Preparacion defensa tesis: diapositivas, demo en vivo y Q&amp;A</t>
+        </is>
+      </c>
+      <c r="E110" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="F110" s="10" t="n">
+        <v>46202</v>
+      </c>
+      <c r="G110" s="10" t="n">
+        <v>46220</v>
+      </c>
+      <c r="H110" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="I110" s="8" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="J110" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="24" customHeight="1">
+      <c r="A111" s="6" t="n"/>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="D111" s="6" t="inlineStr">
+        <is>
+          <t>Revision y aprobacion del asesor: validacion final tesis y sistema</t>
+        </is>
+      </c>
+      <c r="E111" s="9" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="F111" s="10" t="n">
+        <v>46221</v>
+      </c>
+      <c r="G111" s="10" t="n">
+        <v>46233</v>
+      </c>
+      <c r="H111" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="I111" s="8" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="J111" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="24" customHeight="1">
+      <c r="A112" s="6" t="n"/>
+      <c r="B112" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="n">
+        <v>82</v>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>Cierre proyecto: limpieza codigo, README, tag v1.2.0 en git</t>
+        </is>
+      </c>
+      <c r="E112" s="12" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
+      <c r="F112" s="10" t="n">
+        <v>46234</v>
+      </c>
+      <c r="G112" s="10" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H112" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="I112" s="8" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="J112" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="24" customHeight="1">
+      <c r="A113" s="6" t="n"/>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="D113" s="6" t="inlineStr">
+        <is>
+          <t>PDF final de tesis (TESIS_VERIFEX.pdf) con formato definitivo</t>
+        </is>
+      </c>
+      <c r="E113" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="F113" s="10" t="n">
+        <v>46234</v>
+      </c>
+      <c r="G113" s="10" t="n">
+        <v>46253</v>
+      </c>
+      <c r="H113" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I113" s="8" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="J113" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="24" customHeight="1">
+      <c r="A114" s="6" t="n"/>
+      <c r="B114" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C114" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="D114" s="6" t="inlineStr">
+        <is>
+          <t>Revision final y validacion de entrega segun requisitos</t>
+        </is>
+      </c>
+      <c r="E114" s="14" t="inlineStr">
+        <is>
+          <t>Ulises</t>
+        </is>
+      </c>
+      <c r="F114" s="10" t="n">
+        <v>46234</v>
+      </c>
+      <c r="G114" s="10" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H114" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="I114" s="8" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="J114" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="24" customHeight="1">
+      <c r="A115" s="6" t="n"/>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C115" s="8" t="n">
         <v>85</v>
       </c>
-      <c r="D107" s="6" t="inlineStr">
+      <c r="D115" s="6" t="inlineStr">
         <is>
           <t>Pruebas finales de humo y validacion de cierre del proyecto</t>
         </is>
       </c>
-      <c r="E107" s="15" t="inlineStr">
-        <is>
-          <t>Tony</t>
-        </is>
-      </c>
-      <c r="F107" s="10" t="n">
+      <c r="E115" s="13" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="F115" s="10" t="n">
         <v>46234</v>
       </c>
-      <c r="G107" s="10" t="n">
+      <c r="G115" s="10" t="n">
         <v>46254</v>
       </c>
-      <c r="H107" s="8" t="n">
+      <c r="H115" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="I107" s="8" t="inlineStr">
+      <c r="I115" s="8" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="J107" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="24" customHeight="1">
-      <c r="A108" s="16" t="n"/>
-      <c r="B108" s="17" t="inlineStr">
+      <c r="J115" s="11" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="24" customHeight="1">
+      <c r="A116" s="15" t="n"/>
+      <c r="B116" s="16" t="inlineStr">
         <is>
           <t>Iteracion</t>
         </is>
       </c>
-      <c r="C108" s="17" t="inlineStr">
+      <c r="C116" s="16" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="D108" s="16" t="inlineStr">
+      <c r="D116" s="15" t="inlineStr">
         <is>
           <t>v1.2.0 - Tesis completa, sistema VERIFEX version final y presentacion de defensa preparada</t>
         </is>
       </c>
-      <c r="E108" s="17" t="inlineStr">
+      <c r="E116" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F108" s="18" t="n">
+      <c r="F116" s="17" t="n">
         <v>46255</v>
       </c>
-      <c r="G108" s="18" t="n">
+      <c r="G116" s="17" t="n">
         <v>46256</v>
       </c>
-      <c r="H108" s="17" t="n">
+      <c r="H116" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="I108" s="17" t="inlineStr">
+      <c r="I116" s="16" t="inlineStr">
         <is>
           <t>85</t>
         </is>
       </c>
-      <c r="J108" s="17" t="inlineStr">
+      <c r="J116" s="16" t="inlineStr">
         <is>
           <t>Lanzado</t>
         </is>
       </c>
     </row>
-    <row r="109" ht="24" customHeight="1"/>
-    <row r="110" ht="24" customHeight="1"/>
-    <row r="111" ht="24" customHeight="1">
-      <c r="A111" s="20" t="inlineStr">
+    <row r="117" ht="24" customHeight="1"/>
+    <row r="118" ht="24" customHeight="1"/>
+    <row r="119" ht="24" customHeight="1">
+      <c r="A119" s="18" t="inlineStr">
         <is>
           <t>Leyenda:</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="24" customHeight="1">
-      <c r="A112" s="21" t="inlineStr">
+    <row r="120" ht="24" customHeight="1">
+      <c r="A120" s="19" t="inlineStr">
         <is>
           <t>Marco - Backend, frontend, IA, deploy y pruebas</t>
         </is>
       </c>
-      <c r="B112" s="22" t="n"/>
-      <c r="C112" s="22" t="n"/>
-      <c r="D112" s="22" t="n"/>
-    </row>
-    <row r="113" ht="24" customHeight="1">
-      <c r="A113" s="23" t="inlineStr">
+      <c r="B120" s="20" t="n"/>
+      <c r="C120" s="20" t="n"/>
+      <c r="D120" s="20" t="n"/>
+    </row>
+    <row r="121" ht="24" customHeight="1">
+      <c r="A121" s="21" t="inlineStr">
         <is>
           <t>Luis - Frontend, diseno UI/UX y estilos visuales</t>
         </is>
       </c>
-      <c r="B113" s="24" t="n"/>
-      <c r="C113" s="24" t="n"/>
-      <c r="D113" s="24" t="n"/>
-    </row>
-    <row r="114" ht="24" customHeight="1">
-      <c r="A114" s="25" t="inlineStr">
+      <c r="B121" s="22" t="n"/>
+      <c r="C121" s="22" t="n"/>
+      <c r="D121" s="22" t="n"/>
+    </row>
+    <row r="122" ht="24" customHeight="1">
+      <c r="A122" s="23" t="inlineStr">
         <is>
           <t>Ulises - Documentacion y redaccion de tesis</t>
         </is>
       </c>
-      <c r="B114" s="26" t="n"/>
-      <c r="C114" s="26" t="n"/>
-      <c r="D114" s="26" t="n"/>
-    </row>
-    <row r="115" ht="24" customHeight="1">
-      <c r="A115" s="27" t="inlineStr">
-        <is>
-          <t>Tony - Diagramas UML, documentacion y revision de logica</t>
-        </is>
-      </c>
-      <c r="B115" s="28" t="n"/>
-      <c r="C115" s="28" t="n"/>
-      <c r="D115" s="28" t="n"/>
-    </row>
-    <row r="116" ht="24" customHeight="1">
-      <c r="A116" s="29" t="inlineStr">
+      <c r="B122" s="24" t="n"/>
+      <c r="C122" s="24" t="n"/>
+      <c r="D122" s="24" t="n"/>
+    </row>
+    <row r="123" ht="24" customHeight="1">
+      <c r="A123" s="25" t="inlineStr">
         <is>
           <t>★ Iteracion - Hito de lanzamiento de version</t>
         </is>
       </c>
-      <c r="B116" s="30" t="n"/>
-      <c r="C116" s="30" t="n"/>
-      <c r="D116" s="30" t="n"/>
-    </row>
-    <row r="117" ht="24" customHeight="1">
-      <c r="A117" s="29" t="inlineStr">
+      <c r="B123" s="26" t="n"/>
+      <c r="C123" s="26" t="n"/>
+      <c r="D123" s="26" t="n"/>
+    </row>
+    <row r="124" ht="24" customHeight="1">
+      <c r="A124" s="25" t="inlineStr">
         <is>
           <t>Sprint - Tarea individual con duracion definida</t>
         </is>
       </c>
-      <c r="B117" s="30" t="n"/>
-      <c r="C117" s="30" t="n"/>
-      <c r="D117" s="30" t="n"/>
-    </row>
-    <row r="118" ht="24" customHeight="1">
-      <c r="A118" s="29" t="inlineStr">
+      <c r="B124" s="26" t="n"/>
+      <c r="C124" s="26" t="n"/>
+      <c r="D124" s="26" t="n"/>
+    </row>
+    <row r="125" ht="24" customHeight="1">
+      <c r="A125" s="25" t="inlineStr">
         <is>
           <t>Ciclo - Gran fase del proyecto (agrupacion de fases)</t>
         </is>
       </c>
-      <c r="B118" s="30" t="n"/>
-      <c r="C118" s="30" t="n"/>
-      <c r="D118" s="30" t="n"/>
+      <c r="B125" s="26" t="n"/>
+      <c r="C125" s="26" t="n"/>
+      <c r="D125" s="26" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J109"/>
-  <mergeCells count="19">
-    <mergeCell ref="A116:D116"/>
-    <mergeCell ref="A85:J85"/>
+  <autoFilter ref="A1:J116"/>
+  <mergeCells count="18">
+    <mergeCell ref="A120:D120"/>
     <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A112:D112"/>
-    <mergeCell ref="A117:D117"/>
-    <mergeCell ref="A115:D115"/>
-    <mergeCell ref="A114:D114"/>
+    <mergeCell ref="A122:D122"/>
     <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A70:J70"/>
-    <mergeCell ref="A69:J69"/>
+    <mergeCell ref="A124:D124"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A42:J42"/>
+    <mergeCell ref="A91:J91"/>
+    <mergeCell ref="A123:D123"/>
+    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="A125:D125"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A72:J72"/>
+    <mergeCell ref="A121:D121"/>
     <mergeCell ref="A25:J25"/>
+    <mergeCell ref="A90:J90"/>
     <mergeCell ref="A41:J41"/>
-    <mergeCell ref="A118:D118"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A26:J26"/>
-    <mergeCell ref="A113:D113"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A86:J86"/>
-    <mergeCell ref="A42:J42"/>
+    <mergeCell ref="A71:J71"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>